<commit_message>
feat(scheduler): ejecutar jobs en cola secuencial y permitir ejecucion inmediata
- Los jobs que coinciden en la misma hora (movil y escritorio a las 20:00 y
  22:00) se ejecutan uno despues del otro para que dos Chrome no compitan por
  CPU y red y alteren las metricas de Lighthouse.
- `npm run scheduler -- --run-now <jobId|all>` ejecuta jobs por el mismo flujo
  del scheduler y termina; sirve para probarlo y capturar evidencias.
- Las ejecuciones lanzadas por el scheduler se registran con origen
  "scheduler" en data/job-runs.json y en el spreadsheet.
- Se incluye la prueba realizada: dos jobs de prueba programados a las 23:56
  (America/Bogota) se ejecutaron en cola y actualizaron JSON y spreadsheet.
</commit_message>
<xml_diff>
--- a/spreadsheet/metricas-web.xlsx
+++ b/spreadsheet/metricas-web.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="140">
   <si>
     <t>Página</t>
   </si>
@@ -104,202 +104,220 @@
     <t>Isabela Quintero Murillo</t>
   </si>
   <si>
+    <t>2026-10-29 23:56:18</t>
+  </si>
+  <si>
+    <t>prueba-cola-mobile</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:56:46</t>
+  </si>
+  <si>
+    <t>prueba-cola-desktop</t>
+  </si>
+  <si>
+    <t>Última actualización del spreadsheet</t>
+  </si>
+  <si>
+    <t>Job: prueba-cola-desktop (ok)</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Fecha (Bogotá)</t>
+  </si>
+  <si>
+    <t>Timestamp ISO</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:04:08</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:04:08.879Z</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/voluntariado</t>
+  </si>
+  <si>
+    <t>✔ OK</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-10-29 18:04:44</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:04:44.676Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:05:39</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:05:39.937Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:06:08</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:06:08.560Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:08:21</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:08:21.173Z</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/financiacion</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:08:52</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:08:52.270Z</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/internacionalizacion</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:09:20</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:09:20.557Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:10:11</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:10:11.426Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:11:21</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:11:21.270Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:13:57</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:13:57.420Z</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:14:30.367Z</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:14:45.761Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:15:04</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:15:04.038Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:15:32</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:15:32.253Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:16:00</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:16:00.196Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:16:18</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:16:18.800Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:20:57</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:20:57.336Z</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:21:31.745Z</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:21:59.813Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:22:18</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:22:18.156Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:20:52</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:20:52.225Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:21:09</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:21:09.878Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:23:18</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:23:18.570Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:23:28</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:23:28.896Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:52:05</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:52:05.014Z</t>
+  </si>
+  <si>
+    <t>mobile-diario-22</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:52:30</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:52:30.193Z</t>
+  </si>
+  <si>
+    <t>desktop-diario-22</t>
+  </si>
+  <si>
     <t>2026-10-29 23:54:21</t>
   </si>
   <si>
+    <t>2026-10-30T04:54:21.680Z</t>
+  </si>
+  <si>
     <t>mobile-diario-20</t>
   </si>
   <si>
-    <t>2026-10-29 23:52:30</t>
-  </si>
-  <si>
-    <t>desktop-diario-22</t>
-  </si>
-  <si>
-    <t>Última actualización del spreadsheet</t>
-  </si>
-  <si>
-    <t>Job: mobile-diario-20 (ok)</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Fecha (Bogotá)</t>
-  </si>
-  <si>
-    <t>Timestamp ISO</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:04:08</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:04:08.879Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/voluntariado</t>
-  </si>
-  <si>
-    <t>✔ OK</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-10-29 18:04:44</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:04:44.676Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:05:39</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:05:39.937Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:06:08</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:06:08.560Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:08:21</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:08:21.173Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/financiacion</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:08:52</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:08:52.270Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/internacionalizacion</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:09:20</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:09:20.557Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:10:11</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:10:11.426Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:11:21</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:11:21.270Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:13:57</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:13:57.420Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:14:30.367Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:14:45.761Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:15:04</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:15:04.038Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:15:32</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:15:32.253Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:16:00</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:16:00.196Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:16:18</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:16:18.800Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:20:57</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:20:57.336Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:21:31.745Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:21:59.813Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:22:18</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:22:18.156Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:20:52</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:20:52.225Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:21:09</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:21:09.878Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:23:18</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:23:18.570Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:23:28</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:23:28.896Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:52:05</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:52:05.014Z</t>
-  </si>
-  <si>
-    <t>mobile-diario-22</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:52:30.193Z</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:54:21.680Z</t>
+    <t>2026-10-30T04:56:18.862Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:56:46.487Z</t>
   </si>
   <si>
     <t>Perf. promedio móvil</t>
@@ -351,6 +369,18 @@
   </si>
   <si>
     <t>mobile</t>
+  </si>
+  <si>
+    <t>scheduler</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:56:00</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:56:19</t>
+  </si>
+  <si>
+    <t>desktop</t>
   </si>
   <si>
     <t>Métrica</t>
@@ -1098,34 +1128,34 @@
         <v>30</v>
       </c>
       <c r="F6">
-        <v>0.95</v>
+        <v>1.14</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H6">
-        <v>0.98</v>
+        <v>1.17</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J6">
-        <v>2.42</v>
+        <v>2.67</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L6">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="N6">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O6">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1151,13 +1181,13 @@
         <v>20</v>
       </c>
       <c r="H7">
-        <v>1.01</v>
+        <v>0.97</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J7">
-        <v>2.55</v>
+        <v>2.45</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>20</v>
@@ -1169,10 +1199,10 @@
         <v>21</v>
       </c>
       <c r="N7">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O7">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1180,7 +1210,7 @@
         <v>33</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>34</v>
@@ -1195,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2679,13 +2709,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="E27" t="s">
         <v>27</v>
@@ -2735,13 +2765,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="C28" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="E28" t="s">
         <v>27</v>
@@ -2783,6 +2813,118 @@
         <v>44</v>
       </c>
       <c r="R28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" t="s">
+        <v>99</v>
+      </c>
+      <c r="D29" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" t="s">
+        <v>28</v>
+      </c>
+      <c r="G29" t="s">
+        <v>57</v>
+      </c>
+      <c r="H29" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29">
+        <v>1.14</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K29">
+        <v>1.17</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M29">
+        <v>2.67</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O29">
+        <v>96</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>44</v>
+      </c>
+      <c r="R29" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E30" t="s">
+        <v>27</v>
+      </c>
+      <c r="F30" t="s">
+        <v>28</v>
+      </c>
+      <c r="G30" t="s">
+        <v>57</v>
+      </c>
+      <c r="H30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30">
+        <v>0.94</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K30">
+        <v>0.97</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M30">
+        <v>2.45</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O30">
+        <v>85</v>
+      </c>
+      <c r="P30" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>44</v>
+      </c>
+      <c r="R30" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2815,19 +2957,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2884,19 +3026,19 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D4">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="F4">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="G4">
-        <v>1.1</v>
+        <v>1.07</v>
       </c>
     </row>
   </sheetData>
@@ -2908,7 +3050,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2927,28 +3069,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>39</v>
@@ -2956,25 +3098,25 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="E2">
         <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="G2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -2983,6 +3125,70 @@
         <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G3" t="s">
+        <v>117</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3006,7 +3212,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
@@ -3015,49 +3221,49 @@
         <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3065,18 +3271,18 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(evidencias): ejecutar los cuatro jobs y guardar evidencias de informe y spreadsheet
- Se ejecutaron mobile-diario-20, desktop-diario-20, mobile-diario-22 y
  desktop-diario-22 con el scheduler (--run-now all): 12/12 pruebas correctas
  para las tres paginas; JSON, job-runs y spreadsheet actualizados tras cada job.
- evidencias/ incluye capturas del informe web (escritorio y movil), vistas de
  las hojas del spreadsheet y los logs del scheduler (ejecucion de los 4 jobs y
  prueba del cron en cola).
</commit_message>
<xml_diff>
--- a/spreadsheet/metricas-web.xlsx
+++ b/spreadsheet/metricas-web.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="168">
   <si>
     <t>Página</t>
   </si>
@@ -71,253 +71,328 @@
     <t>Moto G4 (412x823)</t>
   </si>
   <si>
+    <t>2026-10-29 23:59:04</t>
+  </si>
+  <si>
+    <t>mobile-diario-22</t>
+  </si>
+  <si>
+    <t>✔ Bueno</t>
+  </si>
+  <si>
+    <t>Desktop (1350x940)</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:59:37</t>
+  </si>
+  <si>
+    <t>desktop-diario-22</t>
+  </si>
+  <si>
+    <t>Financiación de estudios</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:59:14</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:59:50</t>
+  </si>
+  <si>
+    <t>▲ Por mejorar</t>
+  </si>
+  <si>
+    <t>Internacionalización</t>
+  </si>
+  <si>
+    <t>Isabela Quintero Murillo</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:59:24</t>
+  </si>
+  <si>
+    <t>2026-10-30 00:00:01</t>
+  </si>
+  <si>
+    <t>Última actualización del spreadsheet</t>
+  </si>
+  <si>
+    <t>Job: desktop-diario-22 (ok)</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Fecha (Bogotá)</t>
+  </si>
+  <si>
+    <t>Timestamp ISO</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:04:08</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:04:08.879Z</t>
+  </si>
+  <si>
+    <t>sin registro</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/voluntariado</t>
+  </si>
+  <si>
+    <t>✔ OK</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-10-29 18:04:44</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:04:44.676Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:05:39</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:05:39.937Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:06:08</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:06:08.560Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:08:21</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:08:21.173Z</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/financiacion</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:08:52</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:08:52.270Z</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/internacionalizacion</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:09:20</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:09:20.557Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:10:11</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:10:11.426Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:11:21</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:11:21.270Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:13:57</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:13:57.420Z</t>
+  </si>
+  <si>
     <t>2026-10-29 18:14:30</t>
   </si>
   <si>
-    <t>sin registro</t>
-  </si>
-  <si>
-    <t>✔ Bueno</t>
-  </si>
-  <si>
-    <t>▲ Por mejorar</t>
-  </si>
-  <si>
-    <t>Desktop (1350x940)</t>
+    <t>2026-10-29T23:14:30.367Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:14:45</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:14:45.761Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:15:04</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:15:04.038Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:15:32</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:15:32.253Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:16:00</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:16:00.196Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:16:18</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:16:18.800Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:20:57</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:20:57.336Z</t>
   </si>
   <si>
     <t>2026-10-29 18:21:31</t>
   </si>
   <si>
-    <t>Financiación de estudios</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:14:45</t>
+    <t>2026-10-29T23:21:31.745Z</t>
   </si>
   <si>
     <t>2026-10-29 18:21:59</t>
   </si>
   <si>
-    <t>Internacionalización</t>
-  </si>
-  <si>
-    <t>Isabela Quintero Murillo</t>
+    <t>2026-10-29T23:21:59.813Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 18:22:18</t>
+  </si>
+  <si>
+    <t>2026-10-29T23:22:18.156Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:20:52</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:20:52.225Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:21:09</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:21:09.878Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:23:18</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:23:18.570Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:23:28</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:23:28.896Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:52:05</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:52:05.014Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:52:30</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:52:30.193Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:54:21</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:54:21.680Z</t>
+  </si>
+  <si>
+    <t>mobile-diario-20</t>
   </si>
   <si>
     <t>2026-10-29 23:56:18</t>
   </si>
   <si>
+    <t>2026-10-30T04:56:18.862Z</t>
+  </si>
+  <si>
     <t>prueba-cola-mobile</t>
   </si>
   <si>
     <t>2026-10-29 23:56:46</t>
   </si>
   <si>
+    <t>2026-10-30T04:56:46.487Z</t>
+  </si>
+  <si>
     <t>prueba-cola-desktop</t>
   </si>
   <si>
-    <t>Última actualización del spreadsheet</t>
-  </si>
-  <si>
-    <t>Job: prueba-cola-desktop (ok)</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Fecha (Bogotá)</t>
-  </si>
-  <si>
-    <t>Timestamp ISO</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:04:08</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:04:08.879Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/voluntariado</t>
-  </si>
-  <si>
-    <t>✔ OK</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-10-29 18:04:44</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:04:44.676Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:05:39</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:05:39.937Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:06:08</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:06:08.560Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:08:21</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:08:21.173Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/financiacion</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:08:52</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:08:52.270Z</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/internacionalizacion</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:09:20</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:09:20.557Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:10:11</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:10:11.426Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:11:21</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:11:21.270Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:13:57</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:13:57.420Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:14:30.367Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:14:45.761Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:15:04</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:15:04.038Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:15:32</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:15:32.253Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:16:00</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:16:00.196Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:16:18</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:16:18.800Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:20:57</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:20:57.336Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:21:31.745Z</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:21:59.813Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 18:22:18</t>
-  </si>
-  <si>
-    <t>2026-10-29T23:22:18.156Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:20:52</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:20:52.225Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:21:09</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:21:09.878Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:23:18</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:23:18.570Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:23:28</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:23:28.896Z</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:52:05</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:52:05.014Z</t>
-  </si>
-  <si>
-    <t>mobile-diario-22</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:52:30</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:52:30.193Z</t>
-  </si>
-  <si>
-    <t>desktop-diario-22</t>
-  </si>
-  <si>
-    <t>2026-10-29 23:54:21</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:54:21.680Z</t>
-  </si>
-  <si>
-    <t>mobile-diario-20</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:56:18.862Z</t>
-  </si>
-  <si>
-    <t>2026-10-30T04:56:46.487Z</t>
+    <t>2026-10-29 23:57:49</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:57:49.177Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:58:01</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:58:01.622Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:58:12</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:58:12.020Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:58:25</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:58:25.713Z</t>
+  </si>
+  <si>
+    <t>desktop-diario-20</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:58:39</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:58:39.812Z</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:58:50</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:58:50.362Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:59:04.221Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:59:14.445Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:59:24.632Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:59:37.876Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T04:59:50.799Z</t>
+  </si>
+  <si>
+    <t>2026-10-30T05:00:01.026Z</t>
   </si>
   <si>
     <t>Perf. promedio móvil</t>
@@ -381,6 +456,15 @@
   </si>
   <si>
     <t>desktop</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:57:34</t>
+  </si>
+  <si>
+    <t>voluntariado, financiacion, internacionalizacion</t>
+  </si>
+  <si>
+    <t>2026-10-29 23:59:25</t>
   </si>
   <si>
     <t>Métrica</t>
@@ -940,34 +1024,34 @@
         <v>19</v>
       </c>
       <c r="F2">
-        <v>1.41</v>
+        <v>1.09</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H2">
-        <v>1.94</v>
+        <v>1.17</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J2">
-        <v>1.6</v>
+        <v>1.18</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L2">
-        <v>83</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>21</v>
+        <v>98</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="N2">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -978,43 +1062,43 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
       <c r="F3">
-        <v>1.29</v>
+        <v>1.1</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H3">
-        <v>1.81</v>
+        <v>1.13</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J3">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L3">
-        <v>60</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>21</v>
+        <v>95</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="N3">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="O3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1034,34 +1118,34 @@
         <v>19</v>
       </c>
       <c r="F4">
-        <v>1.06</v>
+        <v>0.97</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H4">
-        <v>1.1</v>
+        <v>0.98</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J4">
-        <v>2.68</v>
+        <v>2.19</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L4">
-        <v>73</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>21</v>
+        <v>100</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="N4">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1072,148 +1156,148 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
         <v>26</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F5">
-        <v>1.1</v>
+        <v>0.97</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H5">
-        <v>1.17</v>
+        <v>0.98</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J5">
-        <v>4.6</v>
+        <v>3.59</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="L5">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N5">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="O5">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F6">
-        <v>1.14</v>
+        <v>0.97</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H6">
-        <v>1.17</v>
+        <v>0.98</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J6">
-        <v>2.67</v>
+        <v>2.07</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L6">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="N6">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="O6">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>0.94</v>
+        <v>0.97</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H7">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J7">
-        <v>2.45</v>
+        <v>1.94</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="L7">
-        <v>85</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>21</v>
+        <v>94</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="N7">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="O7">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1225,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1250,13 +1334,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -1268,7 +1352,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -1298,10 +1382,10 @@
         <v>12</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -1309,13 +1393,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>42</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
       </c>
       <c r="E2" t="s">
         <v>15</v>
@@ -1351,7 +1435,7 @@
         <v>71</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q2" t="s">
         <v>44</v>
@@ -1371,7 +1455,7 @@
         <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
@@ -1407,7 +1491,7 @@
         <v>70</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q3" t="s">
         <v>44</v>
@@ -1427,7 +1511,7 @@
         <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
@@ -1463,7 +1547,7 @@
         <v>71</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q4" t="s">
         <v>44</v>
@@ -1483,7 +1567,7 @@
         <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -1519,7 +1603,7 @@
         <v>71</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q5" t="s">
         <v>44</v>
@@ -1539,7 +1623,7 @@
         <v>53</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
         <v>24</v>
@@ -1569,13 +1653,13 @@
         <v>4.91</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O6">
         <v>59</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q6" t="s">
         <v>44</v>
@@ -1595,13 +1679,13 @@
         <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G7" t="s">
         <v>57</v>
@@ -1625,13 +1709,13 @@
         <v>5.48</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O7">
         <v>57</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q7" t="s">
         <v>44</v>
@@ -1651,7 +1735,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
         <v>15</v>
@@ -1687,7 +1771,7 @@
         <v>69</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q8" t="s">
         <v>44</v>
@@ -1707,7 +1791,7 @@
         <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
         <v>24</v>
@@ -1737,13 +1821,13 @@
         <v>4.69</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O9">
         <v>59</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q9" t="s">
         <v>44</v>
@@ -1763,7 +1847,7 @@
         <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>24</v>
@@ -1793,13 +1877,13 @@
         <v>4.81</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O10">
         <v>60</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q10" t="s">
         <v>44</v>
@@ -1819,7 +1903,7 @@
         <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
@@ -1849,13 +1933,13 @@
         <v>3.51</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O11">
         <v>72</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q11" t="s">
         <v>44</v>
@@ -1869,13 +1953,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E12" t="s">
         <v>15</v>
@@ -1911,7 +1995,7 @@
         <v>83</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q12" t="s">
         <v>44</v>
@@ -1925,13 +2009,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E13" t="s">
         <v>24</v>
@@ -1967,7 +2051,7 @@
         <v>73</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q13" t="s">
         <v>44</v>
@@ -1981,19 +2065,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G14" t="s">
         <v>57</v>
@@ -2023,7 +2107,7 @@
         <v>78</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q14" t="s">
         <v>44</v>
@@ -2037,13 +2121,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
         <v>15</v>
@@ -2055,7 +2139,7 @@
         <v>43</v>
       </c>
       <c r="H15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I15">
         <v>1.31</v>
@@ -2079,7 +2163,7 @@
         <v>59</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q15" t="s">
         <v>44</v>
@@ -2093,13 +2177,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
@@ -2111,7 +2195,7 @@
         <v>54</v>
       </c>
       <c r="H16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I16">
         <v>1.11</v>
@@ -2129,13 +2213,13 @@
         <v>4.57</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O16">
         <v>56</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q16" t="s">
         <v>44</v>
@@ -2149,25 +2233,25 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G17" t="s">
         <v>57</v>
       </c>
       <c r="H17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I17">
         <v>1.12</v>
@@ -2191,7 +2275,7 @@
         <v>61</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q17" t="s">
         <v>44</v>
@@ -2205,19 +2289,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G18" t="s">
         <v>57</v>
@@ -2241,13 +2325,13 @@
         <v>3.67</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O18">
         <v>70</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q18" t="s">
         <v>44</v>
@@ -2261,13 +2345,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
         <v>15</v>
@@ -2279,7 +2363,7 @@
         <v>43</v>
       </c>
       <c r="H19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I19">
         <v>1.29</v>
@@ -2303,7 +2387,7 @@
         <v>60</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q19" t="s">
         <v>44</v>
@@ -2317,13 +2401,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E20" t="s">
         <v>24</v>
@@ -2335,7 +2419,7 @@
         <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I20">
         <v>1.1</v>
@@ -2353,13 +2437,13 @@
         <v>4.6</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O20">
         <v>56</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q20" t="s">
         <v>44</v>
@@ -2373,25 +2457,25 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G21" t="s">
         <v>57</v>
       </c>
       <c r="H21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I21">
         <v>1.14</v>
@@ -2415,7 +2499,7 @@
         <v>60</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q21" t="s">
         <v>44</v>
@@ -2429,19 +2513,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G22" t="s">
         <v>57</v>
@@ -2485,25 +2569,25 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G23" t="s">
         <v>57</v>
       </c>
       <c r="H23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I23">
         <v>0.94</v>
@@ -2527,7 +2611,7 @@
         <v>87</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q23" t="s">
         <v>44</v>
@@ -2541,19 +2625,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G24" t="s">
         <v>57</v>
@@ -2597,25 +2681,25 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="E25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G25" t="s">
         <v>57</v>
       </c>
       <c r="H25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I25">
         <v>0.98</v>
@@ -2653,19 +2737,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D26" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="E26" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G26" t="s">
         <v>57</v>
@@ -2709,25 +2793,25 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C27" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="E27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G27" t="s">
         <v>57</v>
       </c>
       <c r="H27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I27">
         <v>0.94</v>
@@ -2751,7 +2835,7 @@
         <v>85</v>
       </c>
       <c r="P27" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q27" t="s">
         <v>44</v>
@@ -2765,19 +2849,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E28" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G28" t="s">
         <v>57</v>
@@ -2821,19 +2905,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E29" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" t="s">
         <v>29</v>
-      </c>
-      <c r="C29" t="s">
-        <v>99</v>
-      </c>
-      <c r="D29" t="s">
-        <v>30</v>
-      </c>
-      <c r="E29" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" t="s">
-        <v>28</v>
       </c>
       <c r="G29" t="s">
         <v>57</v>
@@ -2877,25 +2961,25 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="E30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G30" t="s">
         <v>57</v>
       </c>
       <c r="H30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I30">
         <v>0.94</v>
@@ -2919,12 +3003,684 @@
         <v>85</v>
       </c>
       <c r="P30" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>44</v>
+      </c>
+      <c r="R30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" t="s">
+        <v>100</v>
+      </c>
+      <c r="E31" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" t="s">
+        <v>43</v>
+      </c>
+      <c r="H31" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31">
+        <v>1.09</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K31">
+        <v>1.1</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M31">
+        <v>1.31</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O31">
+        <v>98</v>
+      </c>
+      <c r="P31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>44</v>
+      </c>
+      <c r="R31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" t="s">
+        <v>110</v>
+      </c>
+      <c r="D32" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H32" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32">
+        <v>0.97</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K32">
+        <v>0.98</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M32">
+        <v>2.79</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O32">
+        <v>98</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>44</v>
+      </c>
+      <c r="R32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" t="s">
+        <v>112</v>
+      </c>
+      <c r="D33" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" t="s">
+        <v>57</v>
+      </c>
+      <c r="H33" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33">
+        <v>0.94</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K33">
+        <v>0.95</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M33">
+        <v>1.7</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O33">
+        <v>100</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>44</v>
+      </c>
+      <c r="R33" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" t="s">
+        <v>115</v>
+      </c>
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
+        <v>16</v>
+      </c>
+      <c r="G34" t="s">
+        <v>43</v>
+      </c>
+      <c r="H34" t="s">
         <v>21</v>
       </c>
-      <c r="Q30" t="s">
-        <v>44</v>
-      </c>
-      <c r="R30" t="s">
+      <c r="I34">
+        <v>1.09</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K34">
+        <v>1.17</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M34">
+        <v>1.09</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O34">
+        <v>94</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>44</v>
+      </c>
+      <c r="R34" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>116</v>
+      </c>
+      <c r="C35" t="s">
+        <v>117</v>
+      </c>
+      <c r="D35" t="s">
+        <v>115</v>
+      </c>
+      <c r="E35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" t="s">
+        <v>54</v>
+      </c>
+      <c r="H35" t="s">
+        <v>21</v>
+      </c>
+      <c r="I35">
+        <v>0.97</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K35">
+        <v>1.01</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M35">
+        <v>4.44</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O35">
+        <v>85</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>44</v>
+      </c>
+      <c r="R35" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" t="s">
+        <v>119</v>
+      </c>
+      <c r="D36" t="s">
+        <v>115</v>
+      </c>
+      <c r="E36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" t="s">
+        <v>29</v>
+      </c>
+      <c r="G36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H36" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36">
+        <v>0.94</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K36">
+        <v>0.98</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M36">
+        <v>1.66</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O36">
+        <v>95</v>
+      </c>
+      <c r="P36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>44</v>
+      </c>
+      <c r="R36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>120</v>
+      </c>
+      <c r="D37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" t="s">
+        <v>43</v>
+      </c>
+      <c r="H37" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37">
+        <v>1.09</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K37">
+        <v>1.17</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M37">
+        <v>1.18</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O37">
+        <v>98</v>
+      </c>
+      <c r="P37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>44</v>
+      </c>
+      <c r="R37" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="s">
+        <v>121</v>
+      </c>
+      <c r="D38" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" t="s">
+        <v>54</v>
+      </c>
+      <c r="H38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38">
+        <v>0.97</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K38">
+        <v>0.98</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M38">
+        <v>2.19</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O38">
+        <v>100</v>
+      </c>
+      <c r="P38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>44</v>
+      </c>
+      <c r="R38" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F39" t="s">
+        <v>29</v>
+      </c>
+      <c r="G39" t="s">
+        <v>57</v>
+      </c>
+      <c r="H39" t="s">
+        <v>17</v>
+      </c>
+      <c r="I39">
+        <v>0.97</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K39">
+        <v>0.98</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M39">
+        <v>2.07</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O39">
+        <v>100</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>44</v>
+      </c>
+      <c r="R39" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" t="s">
+        <v>123</v>
+      </c>
+      <c r="D40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" t="s">
+        <v>43</v>
+      </c>
+      <c r="H40" t="s">
+        <v>21</v>
+      </c>
+      <c r="I40">
+        <v>1.1</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K40">
+        <v>1.13</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M40">
+        <v>1.1</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O40">
+        <v>95</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>44</v>
+      </c>
+      <c r="R40" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>26</v>
+      </c>
+      <c r="C41" t="s">
+        <v>124</v>
+      </c>
+      <c r="D41" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" t="s">
+        <v>24</v>
+      </c>
+      <c r="F41" t="s">
+        <v>16</v>
+      </c>
+      <c r="G41" t="s">
+        <v>54</v>
+      </c>
+      <c r="H41" t="s">
+        <v>21</v>
+      </c>
+      <c r="I41">
+        <v>0.97</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K41">
+        <v>0.98</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M41">
+        <v>3.59</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O41">
+        <v>89</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>44</v>
+      </c>
+      <c r="R41" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42" t="s">
+        <v>125</v>
+      </c>
+      <c r="D42" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" t="s">
+        <v>28</v>
+      </c>
+      <c r="F42" t="s">
+        <v>29</v>
+      </c>
+      <c r="G42" t="s">
+        <v>57</v>
+      </c>
+      <c r="H42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I42">
+        <v>0.97</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K42">
+        <v>1.01</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M42">
+        <v>1.94</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O42">
+        <v>94</v>
+      </c>
+      <c r="P42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>44</v>
+      </c>
+      <c r="R42" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2957,19 +3713,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2980,19 +3736,19 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D2">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="E2">
-        <v>-13</v>
+        <v>-2</v>
       </c>
       <c r="F2">
-        <v>1.68</v>
+        <v>1.54</v>
       </c>
       <c r="G2">
-        <v>1.83</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3003,42 +3759,42 @@
         <v>16</v>
       </c>
       <c r="C3">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D3">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="E3">
-        <v>-9</v>
+        <v>-3</v>
       </c>
       <c r="F3">
-        <v>1.56</v>
+        <v>1.39</v>
       </c>
       <c r="G3">
-        <v>1.19</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E4">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="F4">
-        <v>1.26</v>
+        <v>1.2</v>
       </c>
       <c r="G4">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
     </row>
   </sheetData>
@@ -3050,7 +3806,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3069,54 +3825,54 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" t="s">
         <v>98</v>
-      </c>
-      <c r="B2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D2" t="s">
-        <v>96</v>
       </c>
       <c r="E2">
         <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="G2" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -3130,25 +3886,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E3">
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="G3" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -3162,25 +3918,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="E4">
         <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="G4" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -3189,6 +3945,134 @@
         <v>0</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s">
+        <v>148</v>
+      </c>
+      <c r="G5" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>148</v>
+      </c>
+      <c r="G7" t="s">
+        <v>142</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3212,58 +4096,58 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>127</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>156</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>130</v>
+        <v>158</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3271,18 +4155,18 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>139</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(resultados): registrar medicion de verificacion de internacionalizacion
Ejecucion manual del job mobile-diario-20 para la pagina de
internacionalizacion (performance 94) que comprueba que el JSON, el
registro de jobs y el spreadsheet se actualizan automaticamente.
</commit_message>
<xml_diff>
--- a/spreadsheet/metricas-web.xlsx
+++ b/spreadsheet/metricas-web.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="139">
   <si>
     <t>Proyecto de Métricas Web — Universidad Autónoma de Manizales</t>
   </si>
   <si>
-    <t>Última medición por página y dispositivo. Actualizado el 30/10/2026 a las 00:32:14 (hora de Bogotá) por job desktop-diario-22.</t>
+    <t>Última medición por página y dispositivo. Actualizado el 30/10/2026 a las 02:01:37 (hora de Bogotá) por job mobile-diario-20.</t>
   </si>
   <si>
     <t>Página</t>
@@ -128,174 +128,177 @@
     <t>Isabela Quintero Murillo</t>
   </si>
   <si>
+    <t>30/10/2026</t>
+  </si>
+  <si>
+    <t>02:01:12</t>
+  </si>
+  <si>
+    <t>mobile-diario-20</t>
+  </si>
+  <si>
+    <t>00:00:01</t>
+  </si>
+  <si>
+    <t>Convenciones</t>
+  </si>
+  <si>
+    <t>Deficiente</t>
+  </si>
+  <si>
+    <t>Historial de mediciones</t>
+  </si>
+  <si>
+    <t>Todas las ejecuciones registradas en data/results.json. Tiempos en segundos; fecha y hora de Bogotá.</t>
+  </si>
+  <si>
+    <t>N.º</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>18:04:08</t>
+  </si>
+  <si>
+    <t>Sin registro</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/voluntariado</t>
+  </si>
+  <si>
+    <t>Correcta</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>18:04:44</t>
+  </si>
+  <si>
+    <t>18:05:39</t>
+  </si>
+  <si>
+    <t>18:06:08</t>
+  </si>
+  <si>
+    <t>18:08:21</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/financiacion</t>
+  </si>
+  <si>
+    <t>18:08:52</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/internacionalizacion</t>
+  </si>
+  <si>
+    <t>18:09:20</t>
+  </si>
+  <si>
+    <t>18:10:11</t>
+  </si>
+  <si>
+    <t>18:11:21</t>
+  </si>
+  <si>
+    <t>18:13:57</t>
+  </si>
+  <si>
+    <t>18:14:30</t>
+  </si>
+  <si>
+    <t>18:14:45</t>
+  </si>
+  <si>
+    <t>18:15:04</t>
+  </si>
+  <si>
+    <t>18:15:32</t>
+  </si>
+  <si>
+    <t>18:16:00</t>
+  </si>
+  <si>
+    <t>18:16:18</t>
+  </si>
+  <si>
+    <t>18:20:57</t>
+  </si>
+  <si>
+    <t>18:21:31</t>
+  </si>
+  <si>
+    <t>18:21:59</t>
+  </si>
+  <si>
+    <t>18:22:18</t>
+  </si>
+  <si>
+    <t>23:20:52</t>
+  </si>
+  <si>
+    <t>23:21:09</t>
+  </si>
+  <si>
+    <t>23:23:18</t>
+  </si>
+  <si>
+    <t>23:23:28</t>
+  </si>
+  <si>
+    <t>23:52:05</t>
+  </si>
+  <si>
+    <t>23:52:30</t>
+  </si>
+  <si>
+    <t>23:54:21</t>
+  </si>
+  <si>
+    <t>23:56:18</t>
+  </si>
+  <si>
+    <t>prueba-cola-mobile</t>
+  </si>
+  <si>
+    <t>23:56:46</t>
+  </si>
+  <si>
+    <t>prueba-cola-desktop</t>
+  </si>
+  <si>
+    <t>23:57:49</t>
+  </si>
+  <si>
+    <t>23:58:01</t>
+  </si>
+  <si>
+    <t>23:58:12</t>
+  </si>
+  <si>
+    <t>23:58:25</t>
+  </si>
+  <si>
+    <t>desktop-diario-20</t>
+  </si>
+  <si>
+    <t>23:58:39</t>
+  </si>
+  <si>
+    <t>23:58:50</t>
+  </si>
+  <si>
     <t>23:59:24</t>
   </si>
   <si>
-    <t>30/10/2026</t>
-  </si>
-  <si>
-    <t>00:00:01</t>
-  </si>
-  <si>
-    <t>Convenciones</t>
-  </si>
-  <si>
-    <t>Deficiente</t>
-  </si>
-  <si>
-    <t>Historial de mediciones</t>
-  </si>
-  <si>
-    <t>Todas las ejecuciones registradas en data/results.json. Tiempos en segundos; fecha y hora de Bogotá.</t>
-  </si>
-  <si>
-    <t>N.º</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>18:04:08</t>
-  </si>
-  <si>
-    <t>Sin registro</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/voluntariado</t>
-  </si>
-  <si>
-    <t>Correcta</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>18:04:44</t>
-  </si>
-  <si>
-    <t>18:05:39</t>
-  </si>
-  <si>
-    <t>18:06:08</t>
-  </si>
-  <si>
-    <t>18:08:21</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/financiacion</t>
-  </si>
-  <si>
-    <t>18:08:52</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/internacionalizacion</t>
-  </si>
-  <si>
-    <t>18:09:20</t>
-  </si>
-  <si>
-    <t>18:10:11</t>
-  </si>
-  <si>
-    <t>18:11:21</t>
-  </si>
-  <si>
-    <t>18:13:57</t>
-  </si>
-  <si>
-    <t>18:14:30</t>
-  </si>
-  <si>
-    <t>18:14:45</t>
-  </si>
-  <si>
-    <t>18:15:04</t>
-  </si>
-  <si>
-    <t>18:15:32</t>
-  </si>
-  <si>
-    <t>18:16:00</t>
-  </si>
-  <si>
-    <t>18:16:18</t>
-  </si>
-  <si>
-    <t>18:20:57</t>
-  </si>
-  <si>
-    <t>18:21:31</t>
-  </si>
-  <si>
-    <t>18:21:59</t>
-  </si>
-  <si>
-    <t>18:22:18</t>
-  </si>
-  <si>
-    <t>23:20:52</t>
-  </si>
-  <si>
-    <t>23:21:09</t>
-  </si>
-  <si>
-    <t>23:23:18</t>
-  </si>
-  <si>
-    <t>23:23:28</t>
-  </si>
-  <si>
-    <t>23:52:05</t>
-  </si>
-  <si>
-    <t>23:52:30</t>
-  </si>
-  <si>
-    <t>23:54:21</t>
-  </si>
-  <si>
-    <t>mobile-diario-20</t>
-  </si>
-  <si>
-    <t>23:56:18</t>
-  </si>
-  <si>
-    <t>prueba-cola-mobile</t>
-  </si>
-  <si>
-    <t>23:56:46</t>
-  </si>
-  <si>
-    <t>prueba-cola-desktop</t>
-  </si>
-  <si>
-    <t>23:57:49</t>
-  </si>
-  <si>
-    <t>23:58:01</t>
-  </si>
-  <si>
-    <t>23:58:12</t>
-  </si>
-  <si>
-    <t>23:58:25</t>
-  </si>
-  <si>
-    <t>desktop-diario-20</t>
-  </si>
-  <si>
-    <t>23:58:39</t>
-  </si>
-  <si>
-    <t>23:58:50</t>
-  </si>
-  <si>
     <t>Comparación entre dispositivos</t>
   </si>
   <si>
@@ -369,6 +372,12 @@
   </si>
   <si>
     <t>23:59:25</t>
+  </si>
+  <si>
+    <t>02:00:55</t>
+  </si>
+  <si>
+    <t>02:01:13</t>
   </si>
   <si>
     <t>Umbrales de clasificación</t>
@@ -1261,34 +1270,34 @@
         <v>22</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="H9" s="6">
-        <v>0.97</v>
+        <v>0.94</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="6">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="L9" s="6">
-        <v>2.07</v>
+        <v>2.46</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="N9" s="8">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="O9" s="7" t="s">
         <v>26</v>
@@ -1297,7 +1306,7 @@
         <v>88</v>
       </c>
       <c r="Q9" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -1314,10 +1323,10 @@
         <v>28</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>30</v>
@@ -1355,7 +1364,7 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -1370,7 +1379,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1398,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S45"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1415,7 +1424,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1438,7 +1447,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1461,7 +1470,7 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1479,7 +1488,7 @@
         <v>3</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>4</v>
@@ -1512,10 +1521,10 @@
         <v>16</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1526,10 +1535,10 @@
         <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>19</v>
@@ -1538,7 +1547,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>21</v>
@@ -1571,10 +1580,10 @@
         <v>34</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1585,10 +1594,10 @@
         <v>23</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>19</v>
@@ -1597,7 +1606,7 @@
         <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>21</v>
@@ -1630,10 +1639,10 @@
         <v>34</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -1644,10 +1653,10 @@
         <v>23</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>19</v>
@@ -1656,7 +1665,7 @@
         <v>20</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>21</v>
@@ -1689,10 +1698,10 @@
         <v>34</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1703,10 +1712,10 @@
         <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>19</v>
@@ -1715,7 +1724,7 @@
         <v>20</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -1748,10 +1757,10 @@
         <v>34</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -1762,10 +1771,10 @@
         <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>31</v>
@@ -1774,7 +1783,7 @@
         <v>20</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>21</v>
@@ -1807,10 +1816,10 @@
         <v>34</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -1821,10 +1830,10 @@
         <v>23</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>35</v>
@@ -1833,7 +1842,7 @@
         <v>36</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>21</v>
@@ -1866,10 +1875,10 @@
         <v>34</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -1880,10 +1889,10 @@
         <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>19</v>
@@ -1892,7 +1901,7 @@
         <v>20</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>21</v>
@@ -1925,10 +1934,10 @@
         <v>34</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -1939,10 +1948,10 @@
         <v>23</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>31</v>
@@ -1951,7 +1960,7 @@
         <v>20</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>21</v>
@@ -1984,10 +1993,10 @@
         <v>34</v>
       </c>
       <c r="R12" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -1998,10 +2007,10 @@
         <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>31</v>
@@ -2010,7 +2019,7 @@
         <v>20</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>21</v>
@@ -2043,10 +2052,10 @@
         <v>34</v>
       </c>
       <c r="R13" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -2057,10 +2066,10 @@
         <v>23</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>31</v>
@@ -2069,7 +2078,7 @@
         <v>20</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>21</v>
@@ -2102,10 +2111,10 @@
         <v>34</v>
       </c>
       <c r="R14" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -2116,10 +2125,10 @@
         <v>23</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>19</v>
@@ -2128,7 +2137,7 @@
         <v>20</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>21</v>
@@ -2161,10 +2170,10 @@
         <v>34</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -2175,10 +2184,10 @@
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>31</v>
@@ -2187,7 +2196,7 @@
         <v>20</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>21</v>
@@ -2220,10 +2229,10 @@
         <v>34</v>
       </c>
       <c r="R16" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -2234,10 +2243,10 @@
         <v>23</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>35</v>
@@ -2246,7 +2255,7 @@
         <v>36</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>21</v>
@@ -2279,10 +2288,10 @@
         <v>34</v>
       </c>
       <c r="R17" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -2293,10 +2302,10 @@
         <v>23</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>19</v>
@@ -2305,7 +2314,7 @@
         <v>20</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>27</v>
@@ -2338,10 +2347,10 @@
         <v>34</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -2352,10 +2361,10 @@
         <v>23</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>31</v>
@@ -2364,7 +2373,7 @@
         <v>20</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>27</v>
@@ -2397,10 +2406,10 @@
         <v>34</v>
       </c>
       <c r="R19" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -2411,10 +2420,10 @@
         <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>35</v>
@@ -2423,7 +2432,7 @@
         <v>36</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>27</v>
@@ -2456,10 +2465,10 @@
         <v>34</v>
       </c>
       <c r="R20" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -2470,10 +2479,10 @@
         <v>23</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>35</v>
@@ -2482,7 +2491,7 @@
         <v>36</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>21</v>
@@ -2515,10 +2524,10 @@
         <v>34</v>
       </c>
       <c r="R21" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
@@ -2529,10 +2538,10 @@
         <v>23</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>19</v>
@@ -2541,7 +2550,7 @@
         <v>20</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>27</v>
@@ -2574,10 +2583,10 @@
         <v>34</v>
       </c>
       <c r="R22" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
@@ -2588,10 +2597,10 @@
         <v>23</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>31</v>
@@ -2600,7 +2609,7 @@
         <v>20</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>27</v>
@@ -2633,10 +2642,10 @@
         <v>34</v>
       </c>
       <c r="R23" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -2647,10 +2656,10 @@
         <v>23</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>35</v>
@@ -2659,7 +2668,7 @@
         <v>36</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>27</v>
@@ -2692,10 +2701,10 @@
         <v>34</v>
       </c>
       <c r="R24" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -2706,10 +2715,10 @@
         <v>23</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>35</v>
@@ -2718,7 +2727,7 @@
         <v>36</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>21</v>
@@ -2751,10 +2760,10 @@
         <v>26</v>
       </c>
       <c r="R25" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -2765,10 +2774,10 @@
         <v>23</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>35</v>
@@ -2777,7 +2786,7 @@
         <v>36</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>27</v>
@@ -2810,10 +2819,10 @@
         <v>34</v>
       </c>
       <c r="R26" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
@@ -2824,10 +2833,10 @@
         <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>35</v>
@@ -2836,7 +2845,7 @@
         <v>36</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>21</v>
@@ -2869,10 +2878,10 @@
         <v>26</v>
       </c>
       <c r="R27" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -2883,10 +2892,10 @@
         <v>23</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>35</v>
@@ -2895,7 +2904,7 @@
         <v>36</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>27</v>
@@ -2928,10 +2937,10 @@
         <v>26</v>
       </c>
       <c r="R28" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S28" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
@@ -2942,7 +2951,7 @@
         <v>23</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>25</v>
@@ -2954,7 +2963,7 @@
         <v>36</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>21</v>
@@ -2987,10 +2996,10 @@
         <v>26</v>
       </c>
       <c r="R29" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
@@ -3001,7 +3010,7 @@
         <v>23</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>30</v>
@@ -3013,7 +3022,7 @@
         <v>36</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>27</v>
@@ -3046,10 +3055,10 @@
         <v>34</v>
       </c>
       <c r="R30" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -3060,10 +3069,10 @@
         <v>23</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>35</v>
@@ -3072,7 +3081,7 @@
         <v>36</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>21</v>
@@ -3105,10 +3114,10 @@
         <v>26</v>
       </c>
       <c r="R31" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S31" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
@@ -3131,7 +3140,7 @@
         <v>36</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>21</v>
@@ -3164,10 +3173,10 @@
         <v>26</v>
       </c>
       <c r="R32" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S32" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
@@ -3190,7 +3199,7 @@
         <v>36</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>27</v>
@@ -3223,10 +3232,10 @@
         <v>34</v>
       </c>
       <c r="R33" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
@@ -3240,7 +3249,7 @@
         <v>86</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>19</v>
@@ -3249,7 +3258,7 @@
         <v>20</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>21</v>
@@ -3282,10 +3291,10 @@
         <v>26</v>
       </c>
       <c r="R34" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
@@ -3299,7 +3308,7 @@
         <v>87</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>31</v>
@@ -3308,7 +3317,7 @@
         <v>20</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>21</v>
@@ -3341,10 +3350,10 @@
         <v>26</v>
       </c>
       <c r="R35" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S35" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
@@ -3358,7 +3367,7 @@
         <v>88</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>35</v>
@@ -3367,7 +3376,7 @@
         <v>36</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>21</v>
@@ -3400,10 +3409,10 @@
         <v>26</v>
       </c>
       <c r="R36" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
@@ -3426,7 +3435,7 @@
         <v>20</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>27</v>
@@ -3459,10 +3468,10 @@
         <v>26</v>
       </c>
       <c r="R37" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S37" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
@@ -3485,7 +3494,7 @@
         <v>20</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>27</v>
@@ -3518,10 +3527,10 @@
         <v>34</v>
       </c>
       <c r="R38" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
@@ -3544,7 +3553,7 @@
         <v>36</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>27</v>
@@ -3577,10 +3586,10 @@
         <v>26</v>
       </c>
       <c r="R39" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S39" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
@@ -3603,7 +3612,7 @@
         <v>20</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>21</v>
@@ -3636,10 +3645,10 @@
         <v>26</v>
       </c>
       <c r="R40" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
@@ -3662,7 +3671,7 @@
         <v>20</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>21</v>
@@ -3695,10 +3704,10 @@
         <v>26</v>
       </c>
       <c r="R41" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S41" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
@@ -3709,7 +3718,7 @@
         <v>23</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>25</v>
@@ -3721,7 +3730,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>21</v>
@@ -3754,10 +3763,10 @@
         <v>26</v>
       </c>
       <c r="R42" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
@@ -3780,7 +3789,7 @@
         <v>20</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H43" s="4" t="s">
         <v>27</v>
@@ -3813,10 +3822,10 @@
         <v>26</v>
       </c>
       <c r="R43" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S43" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
@@ -3839,7 +3848,7 @@
         <v>20</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>27</v>
@@ -3872,10 +3881,10 @@
         <v>34</v>
       </c>
       <c r="R44" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S44" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
@@ -3883,10 +3892,10 @@
         <v>41</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>30</v>
@@ -3898,7 +3907,7 @@
         <v>36</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H45" s="4" t="s">
         <v>27</v>
@@ -3931,10 +3940,69 @@
         <v>26</v>
       </c>
       <c r="R45" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S45" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A46" s="5">
+        <v>42</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J46" s="6">
+        <v>0.94</v>
+      </c>
+      <c r="K46" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L46" s="6">
+        <v>1.01</v>
+      </c>
+      <c r="M46" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N46" s="6">
+        <v>2.46</v>
+      </c>
+      <c r="O46" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P46" s="8">
+        <v>94</v>
+      </c>
+      <c r="Q46" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R46" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="S46" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -3964,7 +4032,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3975,7 +4043,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3992,19 +4060,19 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4070,7 +4138,7 @@
         <v>-6</v>
       </c>
       <c r="F7" s="6">
-        <v>1.2</v>
+        <v>1.18</v>
       </c>
       <c r="G7" s="6">
         <v>1.05</v>
@@ -4092,7 +4160,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -4106,7 +4174,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4121,7 +4189,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4139,51 +4207,51 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="F5" s="5">
         <v>17</v>
@@ -4201,7 +4269,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -4209,13 +4277,13 @@
         <v>83</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>82</v>
@@ -4236,7 +4304,7 @@
         <v>0</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -4244,13 +4312,13 @@
         <v>85</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>84</v>
@@ -4271,21 +4339,21 @@
         <v>0</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>88</v>
@@ -4294,7 +4362,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -4306,7 +4374,7 @@
         <v>0</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -4314,7 +4382,7 @@
         <v>90</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>23</v>
@@ -4329,7 +4397,7 @@
         <v>38</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>27</v>
@@ -4341,7 +4409,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -4349,7 +4417,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>23</v>
@@ -4358,13 +4426,13 @@
         <v>92</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="F10" s="5">
         <v>34</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>21</v>
@@ -4376,7 +4444,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -4384,22 +4452,22 @@
         <v>30</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F11" s="5">
         <v>36</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>27</v>
@@ -4411,7 +4479,42 @@
         <v>0</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F12" s="5">
+        <v>18</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
+      <c r="J12" s="5">
+        <v>0</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -4440,7 +4543,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4448,7 +4551,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4456,7 +4559,7 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>26</v>
@@ -4465,49 +4568,49 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4515,13 +4618,13 @@
         <v>15</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(evidencias): ejecutar los 4 jobs y actualizar el analisis del README
Agrega el log de la ejecucion de los 4 jobs (12/12 correctas), las 12
mediciones nuevas en el JSON y el spreadsheet, y explica como se verifico
la programacion de las 20:00 y 22:00.
</commit_message>
<xml_diff>
--- a/spreadsheet/metricas-web.xlsx
+++ b/spreadsheet/metricas-web.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="153">
   <si>
     <t>Proyecto de Métricas Web — Universidad Autónoma de Manizales</t>
   </si>
   <si>
-    <t>Última medición por página y dispositivo. Actualizado el 30/10/2026 a las 02:01:37 (hora de Bogotá) por job mobile-diario-20.</t>
+    <t>Última medición por página y dispositivo. Actualizado el 30/10/2026 a las 02:17:21 (hora de Bogotá) por job desktop-diario-22.</t>
   </si>
   <si>
     <t>Página</t>
@@ -86,217 +86,253 @@
     <t>412 x 823</t>
   </si>
   <si>
+    <t>30/10/2026</t>
+  </si>
+  <si>
+    <t>02:16:24</t>
+  </si>
+  <si>
+    <t>mobile-diario-22</t>
+  </si>
+  <si>
+    <t>Bueno</t>
+  </si>
+  <si>
+    <t>Escritorio</t>
+  </si>
+  <si>
+    <t>1350 x 940</t>
+  </si>
+  <si>
+    <t>02:16:59</t>
+  </si>
+  <si>
+    <t>desktop-diario-22</t>
+  </si>
+  <si>
+    <t>Financiación de estudios</t>
+  </si>
+  <si>
+    <t>02:16:36</t>
+  </si>
+  <si>
+    <t>02:17:11</t>
+  </si>
+  <si>
+    <t>Por mejorar</t>
+  </si>
+  <si>
+    <t>Internacionalización</t>
+  </si>
+  <si>
+    <t>Isabela Quintero Murillo</t>
+  </si>
+  <si>
+    <t>02:16:46</t>
+  </si>
+  <si>
+    <t>02:17:21</t>
+  </si>
+  <si>
+    <t>Convenciones</t>
+  </si>
+  <si>
+    <t>Deficiente</t>
+  </si>
+  <si>
+    <t>Historial de mediciones</t>
+  </si>
+  <si>
+    <t>Todas las ejecuciones registradas en data/results.json. Tiempos en segundos; fecha y hora de Bogotá.</t>
+  </si>
+  <si>
+    <t>N.º</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
     <t>29/10/2026</t>
   </si>
   <si>
+    <t>18:04:08</t>
+  </si>
+  <si>
+    <t>Sin registro</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/voluntariado</t>
+  </si>
+  <si>
+    <t>Correcta</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>18:04:44</t>
+  </si>
+  <si>
+    <t>18:05:39</t>
+  </si>
+  <si>
+    <t>18:06:08</t>
+  </si>
+  <si>
+    <t>18:08:21</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/financiacion</t>
+  </si>
+  <si>
+    <t>18:08:52</t>
+  </si>
+  <si>
+    <t>https://www.autonoma.edu.co/internacionalizacion</t>
+  </si>
+  <si>
+    <t>18:09:20</t>
+  </si>
+  <si>
+    <t>18:10:11</t>
+  </si>
+  <si>
+    <t>18:11:21</t>
+  </si>
+  <si>
+    <t>18:13:57</t>
+  </si>
+  <si>
+    <t>18:14:30</t>
+  </si>
+  <si>
+    <t>18:14:45</t>
+  </si>
+  <si>
+    <t>18:15:04</t>
+  </si>
+  <si>
+    <t>18:15:32</t>
+  </si>
+  <si>
+    <t>18:16:00</t>
+  </si>
+  <si>
+    <t>18:16:18</t>
+  </si>
+  <si>
+    <t>18:20:57</t>
+  </si>
+  <si>
+    <t>18:21:31</t>
+  </si>
+  <si>
+    <t>18:21:59</t>
+  </si>
+  <si>
+    <t>18:22:18</t>
+  </si>
+  <si>
+    <t>23:20:52</t>
+  </si>
+  <si>
+    <t>23:21:09</t>
+  </si>
+  <si>
+    <t>23:23:18</t>
+  </si>
+  <si>
+    <t>23:23:28</t>
+  </si>
+  <si>
+    <t>23:52:05</t>
+  </si>
+  <si>
+    <t>23:52:30</t>
+  </si>
+  <si>
+    <t>23:54:21</t>
+  </si>
+  <si>
+    <t>mobile-diario-20</t>
+  </si>
+  <si>
+    <t>23:56:18</t>
+  </si>
+  <si>
+    <t>prueba-cola-mobile</t>
+  </si>
+  <si>
+    <t>23:56:46</t>
+  </si>
+  <si>
+    <t>prueba-cola-desktop</t>
+  </si>
+  <si>
+    <t>23:57:49</t>
+  </si>
+  <si>
+    <t>23:58:01</t>
+  </si>
+  <si>
+    <t>23:58:12</t>
+  </si>
+  <si>
+    <t>23:58:25</t>
+  </si>
+  <si>
+    <t>desktop-diario-20</t>
+  </si>
+  <si>
+    <t>23:58:39</t>
+  </si>
+  <si>
+    <t>23:58:50</t>
+  </si>
+  <si>
     <t>23:59:04</t>
   </si>
   <si>
-    <t>mobile-diario-22</t>
-  </si>
-  <si>
-    <t>Bueno</t>
-  </si>
-  <si>
-    <t>Escritorio</t>
-  </si>
-  <si>
-    <t>1350 x 940</t>
+    <t>23:59:14</t>
+  </si>
+  <si>
+    <t>23:59:24</t>
   </si>
   <si>
     <t>23:59:37</t>
   </si>
   <si>
-    <t>desktop-diario-22</t>
-  </si>
-  <si>
-    <t>Financiación de estudios</t>
-  </si>
-  <si>
-    <t>23:59:14</t>
-  </si>
-  <si>
     <t>23:59:50</t>
   </si>
   <si>
-    <t>Por mejorar</t>
-  </si>
-  <si>
-    <t>Internacionalización</t>
-  </si>
-  <si>
-    <t>Isabela Quintero Murillo</t>
-  </si>
-  <si>
-    <t>30/10/2026</t>
+    <t>00:00:01</t>
   </si>
   <si>
     <t>02:01:12</t>
   </si>
   <si>
-    <t>mobile-diario-20</t>
-  </si>
-  <si>
-    <t>00:00:01</t>
-  </si>
-  <si>
-    <t>Convenciones</t>
-  </si>
-  <si>
-    <t>Deficiente</t>
-  </si>
-  <si>
-    <t>Historial de mediciones</t>
-  </si>
-  <si>
-    <t>Todas las ejecuciones registradas en data/results.json. Tiempos en segundos; fecha y hora de Bogotá.</t>
-  </si>
-  <si>
-    <t>N.º</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>18:04:08</t>
-  </si>
-  <si>
-    <t>Sin registro</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/voluntariado</t>
-  </si>
-  <si>
-    <t>Correcta</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>18:04:44</t>
-  </si>
-  <si>
-    <t>18:05:39</t>
-  </si>
-  <si>
-    <t>18:06:08</t>
-  </si>
-  <si>
-    <t>18:08:21</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/financiacion</t>
-  </si>
-  <si>
-    <t>18:08:52</t>
-  </si>
-  <si>
-    <t>https://www.autonoma.edu.co/internacionalizacion</t>
-  </si>
-  <si>
-    <t>18:09:20</t>
-  </si>
-  <si>
-    <t>18:10:11</t>
-  </si>
-  <si>
-    <t>18:11:21</t>
-  </si>
-  <si>
-    <t>18:13:57</t>
-  </si>
-  <si>
-    <t>18:14:30</t>
-  </si>
-  <si>
-    <t>18:14:45</t>
-  </si>
-  <si>
-    <t>18:15:04</t>
-  </si>
-  <si>
-    <t>18:15:32</t>
-  </si>
-  <si>
-    <t>18:16:00</t>
-  </si>
-  <si>
-    <t>18:16:18</t>
-  </si>
-  <si>
-    <t>18:20:57</t>
-  </si>
-  <si>
-    <t>18:21:31</t>
-  </si>
-  <si>
-    <t>18:21:59</t>
-  </si>
-  <si>
-    <t>18:22:18</t>
-  </si>
-  <si>
-    <t>23:20:52</t>
-  </si>
-  <si>
-    <t>23:21:09</t>
-  </si>
-  <si>
-    <t>23:23:18</t>
-  </si>
-  <si>
-    <t>23:23:28</t>
-  </si>
-  <si>
-    <t>23:52:05</t>
-  </si>
-  <si>
-    <t>23:52:30</t>
-  </si>
-  <si>
-    <t>23:54:21</t>
-  </si>
-  <si>
-    <t>23:56:18</t>
-  </si>
-  <si>
-    <t>prueba-cola-mobile</t>
-  </si>
-  <si>
-    <t>23:56:46</t>
-  </si>
-  <si>
-    <t>prueba-cola-desktop</t>
-  </si>
-  <si>
-    <t>23:57:49</t>
-  </si>
-  <si>
-    <t>23:58:01</t>
-  </si>
-  <si>
-    <t>23:58:12</t>
-  </si>
-  <si>
-    <t>23:58:25</t>
-  </si>
-  <si>
-    <t>desktop-diario-20</t>
-  </si>
-  <si>
-    <t>23:58:39</t>
-  </si>
-  <si>
-    <t>23:58:50</t>
-  </si>
-  <si>
-    <t>23:59:24</t>
+    <t>02:15:12</t>
+  </si>
+  <si>
+    <t>02:15:24</t>
+  </si>
+  <si>
+    <t>02:15:34</t>
+  </si>
+  <si>
+    <t>02:15:49</t>
+  </si>
+  <si>
+    <t>02:16:01</t>
+  </si>
+  <si>
+    <t>02:16:11</t>
   </si>
   <si>
     <t>Comparación entre dispositivos</t>
@@ -378,6 +414,12 @@
   </si>
   <si>
     <t>02:01:13</t>
+  </si>
+  <si>
+    <t>02:14:58</t>
+  </si>
+  <si>
+    <t>02:15:35</t>
   </si>
   <si>
     <t>Umbrales de clasificación</t>
@@ -564,9 +606,6 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -579,6 +618,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1067,34 +1109,34 @@
         <v>25</v>
       </c>
       <c r="H5" s="6">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J5" s="6">
-        <v>1.17</v>
+        <v>1.13</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>26</v>
       </c>
       <c r="L5" s="6">
-        <v>1.18</v>
+        <v>1.21</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>26</v>
       </c>
       <c r="N5" s="8">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="O5" s="7" t="s">
         <v>26</v>
       </c>
       <c r="P5" s="9">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="Q5" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -1138,16 +1180,16 @@
         <v>26</v>
       </c>
       <c r="N6" s="8">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>26</v>
       </c>
       <c r="P6" s="9">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="Q6" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1173,34 +1215,34 @@
         <v>25</v>
       </c>
       <c r="H7" s="6">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J7" s="6">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>26</v>
       </c>
       <c r="L7" s="6">
-        <v>2.19</v>
+        <v>3.17</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>26</v>
       </c>
       <c r="N7" s="8">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O7" s="7" t="s">
         <v>26</v>
       </c>
       <c r="P7" s="9">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="Q7" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1226,34 +1268,34 @@
         <v>30</v>
       </c>
       <c r="H8" s="6">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J8" s="6">
-        <v>0.98</v>
+        <v>1.03</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="10">
-        <v>3.59</v>
-      </c>
-      <c r="M8" s="11" t="s">
+      <c r="L8" s="6">
+        <v>3.26</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N8" s="9">
+        <v>84</v>
+      </c>
+      <c r="O8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="N8" s="9">
-        <v>89</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>34</v>
-      </c>
       <c r="P8" s="9">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Q8" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1270,43 +1312,43 @@
         <v>22</v>
       </c>
       <c r="E9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>38</v>
-      </c>
       <c r="G9" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="H9" s="6">
-        <v>0.94</v>
+        <v>0.95</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="6">
-        <v>1.01</v>
+        <v>0.96</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="L9" s="6">
-        <v>2.46</v>
+        <v>1.65</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>26</v>
       </c>
       <c r="N9" s="8">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="O9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="P9" s="9">
-        <v>88</v>
+      <c r="P9" s="8">
+        <v>90</v>
       </c>
       <c r="Q9" s="5">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -1323,28 +1365,28 @@
         <v>28</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H10" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="6">
         <v>0.97</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J10" s="6">
-        <v>1.01</v>
-      </c>
       <c r="K10" s="7" t="s">
         <v>26</v>
       </c>
       <c r="L10" s="6">
-        <v>1.94</v>
+        <v>1.84</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>26</v>
@@ -1356,30 +1398,30 @@
         <v>26</v>
       </c>
       <c r="P10" s="9">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q10" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>41</v>
+      <c r="A12" s="11" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="13" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
-        <v>42</v>
+      <c r="A15" s="14" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1398,7 +1440,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:S58"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1424,7 +1466,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1447,7 +1489,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1470,7 +1512,7 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1488,7 +1530,7 @@
         <v>3</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>4</v>
@@ -1521,10 +1563,10 @@
         <v>16</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1532,13 +1574,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>19</v>
@@ -1547,7 +1589,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>21</v>
@@ -1576,14 +1618,14 @@
       <c r="P5" s="9">
         <v>71</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q5" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S5" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1591,13 +1633,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>19</v>
@@ -1606,7 +1648,7 @@
         <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>21</v>
@@ -1635,14 +1677,14 @@
       <c r="P6" s="9">
         <v>70</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -1650,13 +1692,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>19</v>
@@ -1665,7 +1707,7 @@
         <v>20</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>21</v>
@@ -1694,14 +1736,14 @@
       <c r="P7" s="9">
         <v>71</v>
       </c>
-      <c r="Q7" s="11" t="s">
+      <c r="Q7" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S7" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1709,13 +1751,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>19</v>
@@ -1724,7 +1766,7 @@
         <v>20</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -1753,14 +1795,14 @@
       <c r="P8" s="9">
         <v>71</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Q8" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -1768,13 +1810,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>31</v>
@@ -1783,7 +1825,7 @@
         <v>20</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>21</v>
@@ -1803,23 +1845,23 @@
       <c r="M9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N9" s="10">
+      <c r="N9" s="15">
         <v>4.91</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="O9" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P9" s="9">
         <v>59</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="Q9" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S9" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -1827,13 +1869,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>35</v>
@@ -1842,7 +1884,7 @@
         <v>36</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>21</v>
@@ -1862,23 +1904,23 @@
       <c r="M10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N10" s="10">
+      <c r="N10" s="15">
         <v>5.48</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P10" s="9">
         <v>57</v>
       </c>
-      <c r="Q10" s="11" t="s">
+      <c r="Q10" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S10" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S10" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -1886,13 +1928,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>19</v>
@@ -1901,7 +1943,7 @@
         <v>20</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>21</v>
@@ -1930,14 +1972,14 @@
       <c r="P11" s="9">
         <v>69</v>
       </c>
-      <c r="Q11" s="11" t="s">
+      <c r="Q11" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S11" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S11" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -1945,13 +1987,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>31</v>
@@ -1960,7 +2002,7 @@
         <v>20</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>21</v>
@@ -1980,23 +2022,23 @@
       <c r="M12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N12" s="10">
+      <c r="N12" s="15">
         <v>4.69</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="O12" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P12" s="9">
         <v>59</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S12" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -2004,13 +2046,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>31</v>
@@ -2019,7 +2061,7 @@
         <v>20</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>21</v>
@@ -2039,23 +2081,23 @@
       <c r="M13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="10">
+      <c r="N13" s="15">
         <v>4.81</v>
       </c>
-      <c r="O13" s="11" t="s">
+      <c r="O13" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P13" s="9">
         <v>60</v>
       </c>
-      <c r="Q13" s="11" t="s">
+      <c r="Q13" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S13" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S13" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -2063,13 +2105,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>31</v>
@@ -2078,7 +2120,7 @@
         <v>20</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>21</v>
@@ -2098,23 +2140,23 @@
       <c r="M14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="10">
+      <c r="N14" s="15">
         <v>3.51</v>
       </c>
-      <c r="O14" s="11" t="s">
+      <c r="O14" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P14" s="9">
         <v>72</v>
       </c>
-      <c r="Q14" s="11" t="s">
+      <c r="Q14" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R14" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S14" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S14" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -2122,13 +2164,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>19</v>
@@ -2137,7 +2179,7 @@
         <v>20</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>21</v>
@@ -2166,14 +2208,14 @@
       <c r="P15" s="9">
         <v>83</v>
       </c>
-      <c r="Q15" s="11" t="s">
+      <c r="Q15" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S15" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S15" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -2181,13 +2223,13 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>31</v>
@@ -2196,7 +2238,7 @@
         <v>20</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>21</v>
@@ -2225,14 +2267,14 @@
       <c r="P16" s="9">
         <v>73</v>
       </c>
-      <c r="Q16" s="11" t="s">
+      <c r="Q16" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S16" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S16" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -2240,13 +2282,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>35</v>
@@ -2255,7 +2297,7 @@
         <v>36</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>21</v>
@@ -2284,14 +2326,14 @@
       <c r="P17" s="9">
         <v>78</v>
       </c>
-      <c r="Q17" s="11" t="s">
+      <c r="Q17" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R17" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S17" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S17" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -2299,13 +2341,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>19</v>
@@ -2314,7 +2356,7 @@
         <v>20</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>27</v>
@@ -2343,14 +2385,14 @@
       <c r="P18" s="9">
         <v>59</v>
       </c>
-      <c r="Q18" s="11" t="s">
+      <c r="Q18" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S18" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -2358,13 +2400,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>31</v>
@@ -2373,7 +2415,7 @@
         <v>20</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>27</v>
@@ -2393,23 +2435,23 @@
       <c r="M19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N19" s="10">
+      <c r="N19" s="15">
         <v>4.57</v>
       </c>
-      <c r="O19" s="11" t="s">
+      <c r="O19" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P19" s="9">
         <v>56</v>
       </c>
-      <c r="Q19" s="11" t="s">
+      <c r="Q19" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S19" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S19" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -2417,13 +2459,13 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>35</v>
@@ -2432,7 +2474,7 @@
         <v>36</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>27</v>
@@ -2461,14 +2503,14 @@
       <c r="P20" s="9">
         <v>61</v>
       </c>
-      <c r="Q20" s="11" t="s">
+      <c r="Q20" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S20" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S20" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -2476,13 +2518,13 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>35</v>
@@ -2491,7 +2533,7 @@
         <v>36</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>21</v>
@@ -2511,23 +2553,23 @@
       <c r="M21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N21" s="10">
+      <c r="N21" s="15">
         <v>3.67</v>
       </c>
-      <c r="O21" s="11" t="s">
+      <c r="O21" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P21" s="9">
         <v>70</v>
       </c>
-      <c r="Q21" s="11" t="s">
+      <c r="Q21" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S21" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S21" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
@@ -2535,13 +2577,13 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>19</v>
@@ -2550,7 +2592,7 @@
         <v>20</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>27</v>
@@ -2579,14 +2621,14 @@
       <c r="P22" s="9">
         <v>60</v>
       </c>
-      <c r="Q22" s="11" t="s">
+      <c r="Q22" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S22" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S22" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
@@ -2594,13 +2636,13 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>31</v>
@@ -2609,7 +2651,7 @@
         <v>20</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>27</v>
@@ -2629,23 +2671,23 @@
       <c r="M23" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N23" s="10">
+      <c r="N23" s="15">
         <v>4.6</v>
       </c>
-      <c r="O23" s="11" t="s">
+      <c r="O23" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P23" s="9">
         <v>56</v>
       </c>
-      <c r="Q23" s="11" t="s">
+      <c r="Q23" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R23" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S23" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S23" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -2653,13 +2695,13 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>35</v>
@@ -2668,7 +2710,7 @@
         <v>36</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>27</v>
@@ -2697,14 +2739,14 @@
       <c r="P24" s="9">
         <v>60</v>
       </c>
-      <c r="Q24" s="11" t="s">
+      <c r="Q24" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S24" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S24" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -2712,13 +2754,13 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>35</v>
@@ -2727,7 +2769,7 @@
         <v>36</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>21</v>
@@ -2760,10 +2802,10 @@
         <v>26</v>
       </c>
       <c r="R25" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S25" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S25" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -2771,13 +2813,13 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>35</v>
@@ -2786,7 +2828,7 @@
         <v>36</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>27</v>
@@ -2815,14 +2857,14 @@
       <c r="P26" s="9">
         <v>87</v>
       </c>
-      <c r="Q26" s="11" t="s">
+      <c r="Q26" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R26" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S26" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S26" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
@@ -2830,13 +2872,13 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>35</v>
@@ -2845,7 +2887,7 @@
         <v>36</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>21</v>
@@ -2878,10 +2920,10 @@
         <v>26</v>
       </c>
       <c r="R27" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S27" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S27" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -2889,13 +2931,13 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>35</v>
@@ -2904,7 +2946,7 @@
         <v>36</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>27</v>
@@ -2937,10 +2979,10 @@
         <v>26</v>
       </c>
       <c r="R28" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S28" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S28" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
@@ -2948,10 +2990,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>25</v>
@@ -2963,7 +3005,7 @@
         <v>36</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>21</v>
@@ -2996,10 +3038,10 @@
         <v>26</v>
       </c>
       <c r="R29" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S29" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S29" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
@@ -3007,10 +3049,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>30</v>
@@ -3022,7 +3064,7 @@
         <v>36</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>27</v>
@@ -3051,14 +3093,14 @@
       <c r="P30" s="9">
         <v>85</v>
       </c>
-      <c r="Q30" s="11" t="s">
+      <c r="Q30" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R30" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S30" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S30" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -3066,13 +3108,13 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C31" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>35</v>
@@ -3081,7 +3123,7 @@
         <v>36</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>21</v>
@@ -3114,10 +3156,10 @@
         <v>26</v>
       </c>
       <c r="R31" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S31" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S31" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
@@ -3125,7 +3167,7 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>82</v>
@@ -3140,7 +3182,7 @@
         <v>36</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>21</v>
@@ -3173,10 +3215,10 @@
         <v>26</v>
       </c>
       <c r="R32" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S32" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S32" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
@@ -3184,7 +3226,7 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>84</v>
@@ -3199,7 +3241,7 @@
         <v>36</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>27</v>
@@ -3228,14 +3270,14 @@
       <c r="P33" s="9">
         <v>85</v>
       </c>
-      <c r="Q33" s="11" t="s">
+      <c r="Q33" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R33" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S33" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S33" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
@@ -3243,13 +3285,13 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>86</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>19</v>
@@ -3258,7 +3300,7 @@
         <v>20</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>21</v>
@@ -3291,10 +3333,10 @@
         <v>26</v>
       </c>
       <c r="R34" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S34" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S34" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
@@ -3302,13 +3344,13 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>31</v>
@@ -3317,7 +3359,7 @@
         <v>20</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>21</v>
@@ -3350,10 +3392,10 @@
         <v>26</v>
       </c>
       <c r="R35" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S35" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S35" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
@@ -3361,13 +3403,13 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>88</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>35</v>
@@ -3376,7 +3418,7 @@
         <v>36</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>21</v>
@@ -3409,10 +3451,10 @@
         <v>26</v>
       </c>
       <c r="R36" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S36" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S36" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
@@ -3420,7 +3462,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>89</v>
@@ -3435,7 +3477,7 @@
         <v>20</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>27</v>
@@ -3468,10 +3510,10 @@
         <v>26</v>
       </c>
       <c r="R37" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S37" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S37" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
@@ -3479,7 +3521,7 @@
         <v>34</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>91</v>
@@ -3494,7 +3536,7 @@
         <v>20</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>27</v>
@@ -3514,23 +3556,23 @@
       <c r="M38" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N38" s="10">
+      <c r="N38" s="15">
         <v>4.44</v>
       </c>
-      <c r="O38" s="11" t="s">
+      <c r="O38" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P38" s="9">
         <v>85</v>
       </c>
-      <c r="Q38" s="11" t="s">
+      <c r="Q38" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R38" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S38" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S38" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
@@ -3538,7 +3580,7 @@
         <v>35</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>92</v>
@@ -3553,7 +3595,7 @@
         <v>36</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>27</v>
@@ -3586,10 +3628,10 @@
         <v>26</v>
       </c>
       <c r="R39" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S39" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S39" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
@@ -3597,10 +3639,10 @@
         <v>36</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>25</v>
@@ -3612,7 +3654,7 @@
         <v>20</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>21</v>
@@ -3645,10 +3687,10 @@
         <v>26</v>
       </c>
       <c r="R40" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S40" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S40" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
@@ -3656,10 +3698,10 @@
         <v>37</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>25</v>
@@ -3671,7 +3713,7 @@
         <v>20</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>21</v>
@@ -3704,10 +3746,10 @@
         <v>26</v>
       </c>
       <c r="R41" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S41" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S41" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
@@ -3715,10 +3757,10 @@
         <v>38</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>25</v>
@@ -3730,7 +3772,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>21</v>
@@ -3763,10 +3805,10 @@
         <v>26</v>
       </c>
       <c r="R42" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S42" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S42" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
@@ -3774,10 +3816,10 @@
         <v>39</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>30</v>
@@ -3789,7 +3831,7 @@
         <v>20</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H43" s="4" t="s">
         <v>27</v>
@@ -3822,10 +3864,10 @@
         <v>26</v>
       </c>
       <c r="R43" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S43" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S43" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
@@ -3833,10 +3875,10 @@
         <v>40</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>30</v>
@@ -3848,7 +3890,7 @@
         <v>20</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>27</v>
@@ -3868,23 +3910,23 @@
       <c r="M44" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N44" s="10">
+      <c r="N44" s="15">
         <v>3.59</v>
       </c>
-      <c r="O44" s="11" t="s">
+      <c r="O44" s="10" t="s">
         <v>34</v>
       </c>
       <c r="P44" s="9">
         <v>89</v>
       </c>
-      <c r="Q44" s="11" t="s">
+      <c r="Q44" s="10" t="s">
         <v>34</v>
       </c>
       <c r="R44" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S44" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S44" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
@@ -3892,10 +3934,10 @@
         <v>41</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>30</v>
@@ -3907,7 +3949,7 @@
         <v>36</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H45" s="4" t="s">
         <v>27</v>
@@ -3940,10 +3982,10 @@
         <v>26</v>
       </c>
       <c r="R45" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S45" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="S45" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
@@ -3951,13 +3993,13 @@
         <v>42</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>35</v>
@@ -3966,7 +4008,7 @@
         <v>36</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H46" s="4" t="s">
         <v>21</v>
@@ -3999,10 +4041,718 @@
         <v>26</v>
       </c>
       <c r="R46" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S46" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="S46" s="4" t="s">
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A47" s="5">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J47" s="6">
+        <v>1.11</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L47" s="6">
+        <v>1.12</v>
+      </c>
+      <c r="M47" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N47" s="6">
+        <v>1.19</v>
+      </c>
+      <c r="O47" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P47" s="8">
+        <v>99</v>
+      </c>
+      <c r="Q47" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R47" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S47" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J48" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="K48" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L48" s="6">
+        <v>1</v>
+      </c>
+      <c r="M48" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N48" s="6">
+        <v>2.3</v>
+      </c>
+      <c r="O48" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P48" s="8">
+        <v>97</v>
+      </c>
+      <c r="Q48" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R48" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S48" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A49" s="5">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J49" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L49" s="6">
+        <v>0.96</v>
+      </c>
+      <c r="M49" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N49" s="6">
+        <v>2.1</v>
+      </c>
+      <c r="O49" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P49" s="8">
+        <v>98</v>
+      </c>
+      <c r="Q49" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R49" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S49" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
+        <v>46</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J50" s="6">
+        <v>1.1</v>
+      </c>
+      <c r="K50" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L50" s="6">
+        <v>1.13</v>
+      </c>
+      <c r="M50" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N50" s="6">
+        <v>1.1</v>
+      </c>
+      <c r="O50" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P50" s="8">
+        <v>92</v>
+      </c>
+      <c r="Q50" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R50" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S50" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>47</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J51" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="K51" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L51" s="6">
+        <v>1.02</v>
+      </c>
+      <c r="M51" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N51" s="6">
+        <v>2.18</v>
+      </c>
+      <c r="O51" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P51" s="9">
+        <v>87</v>
+      </c>
+      <c r="Q51" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="R51" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S51" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>48</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="K52" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L52" s="6">
+        <v>0.99</v>
+      </c>
+      <c r="M52" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N52" s="6">
+        <v>1.85</v>
+      </c>
+      <c r="O52" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P52" s="8">
+        <v>92</v>
+      </c>
+      <c r="Q52" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R52" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S52" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>49</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J53" s="6">
+        <v>1.1</v>
+      </c>
+      <c r="K53" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L53" s="6">
+        <v>1.13</v>
+      </c>
+      <c r="M53" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N53" s="6">
+        <v>1.21</v>
+      </c>
+      <c r="O53" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P53" s="8">
+        <v>99</v>
+      </c>
+      <c r="Q53" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R53" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S53" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>50</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J54" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="K54" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L54" s="6">
+        <v>0.99</v>
+      </c>
+      <c r="M54" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N54" s="6">
+        <v>3.17</v>
+      </c>
+      <c r="O54" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P54" s="8">
+        <v>97</v>
+      </c>
+      <c r="Q54" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R54" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S54" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>51</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J55" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="K55" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L55" s="6">
+        <v>0.96</v>
+      </c>
+      <c r="M55" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N55" s="6">
+        <v>1.65</v>
+      </c>
+      <c r="O55" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P55" s="8">
+        <v>99</v>
+      </c>
+      <c r="Q55" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R55" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S55" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>52</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J56" s="6">
+        <v>1.1</v>
+      </c>
+      <c r="K56" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L56" s="6">
+        <v>1.13</v>
+      </c>
+      <c r="M56" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N56" s="6">
+        <v>1.1</v>
+      </c>
+      <c r="O56" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P56" s="8">
+        <v>94</v>
+      </c>
+      <c r="Q56" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R56" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S56" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
         <v>53</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J57" s="6">
+        <v>0.96</v>
+      </c>
+      <c r="K57" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L57" s="6">
+        <v>1.03</v>
+      </c>
+      <c r="M57" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N57" s="6">
+        <v>3.26</v>
+      </c>
+      <c r="O57" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P57" s="9">
+        <v>84</v>
+      </c>
+      <c r="Q57" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="R57" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S57" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A58" s="5">
+        <v>54</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I58" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J58" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="K58" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L58" s="6">
+        <v>0.97</v>
+      </c>
+      <c r="M58" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N58" s="6">
+        <v>1.84</v>
+      </c>
+      <c r="O58" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P58" s="8">
+        <v>94</v>
+      </c>
+      <c r="Q58" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R58" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="S58" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -4032,7 +4782,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4043,7 +4793,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4060,19 +4810,19 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4083,19 +4833,19 @@
         <v>20</v>
       </c>
       <c r="C5" s="9">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D5" s="9">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E5" s="16">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F5" s="6">
-        <v>1.54</v>
+        <v>1.46</v>
       </c>
       <c r="G5" s="6">
-        <v>1.49</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -4106,19 +4856,19 @@
         <v>20</v>
       </c>
       <c r="C6" s="9">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D6" s="9">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E6" s="16">
         <v>-3</v>
       </c>
       <c r="F6" s="6">
-        <v>1.39</v>
+        <v>1.3</v>
       </c>
       <c r="G6" s="6">
-        <v>1.09</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4128,20 +4878,20 @@
       <c r="B7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="9">
-        <v>88</v>
+      <c r="C7" s="8">
+        <v>90</v>
       </c>
       <c r="D7" s="9">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E7" s="16">
         <v>-6</v>
       </c>
       <c r="F7" s="6">
-        <v>1.18</v>
+        <v>1.15</v>
       </c>
       <c r="G7" s="6">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
     </row>
   </sheetData>
@@ -4160,7 +4910,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -4174,7 +4924,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4189,7 +4939,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4207,51 +4957,51 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F5" s="5">
         <v>17</v>
@@ -4269,7 +5019,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -4277,13 +5027,13 @@
         <v>83</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>82</v>
@@ -4304,7 +5054,7 @@
         <v>0</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -4312,13 +5062,13 @@
         <v>85</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>84</v>
@@ -4339,21 +5089,21 @@
         <v>0</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>88</v>
@@ -4362,7 +5112,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -4374,7 +5124,7 @@
         <v>0</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -4382,10 +5132,10 @@
         <v>90</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>88</v>
@@ -4397,7 +5147,7 @@
         <v>38</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>27</v>
@@ -4409,7 +5159,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -4417,22 +5167,22 @@
         <v>25</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>92</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F10" s="5">
         <v>34</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>21</v>
@@ -4444,7 +5194,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -4452,22 +5202,22 @@
         <v>30</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="F11" s="5">
         <v>36</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>27</v>
@@ -4479,24 +5229,24 @@
         <v>0</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="F12" s="5">
         <v>18</v>
@@ -4514,7 +5264,147 @@
         <v>0</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F13" s="5">
+        <v>36</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" s="5">
+        <v>3</v>
+      </c>
+      <c r="J13" s="5">
+        <v>0</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F14" s="5">
+        <v>36</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="5">
+        <v>3</v>
+      </c>
+      <c r="J14" s="5">
+        <v>0</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="5">
+        <v>35</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" s="5">
+        <v>3</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="5">
+        <v>35</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="5">
+        <v>3</v>
+      </c>
+      <c r="J16" s="5">
+        <v>0</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -4543,7 +5433,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4551,7 +5441,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4559,7 +5449,7 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>26</v>
@@ -4568,49 +5458,49 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>126</v>
+        <v>139</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>140</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>130</v>
+        <v>143</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>144</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>148</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4618,13 +5508,13 @@
         <v>15</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>137</v>
+        <v>150</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>151</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>